<commit_message>
docs: update stage column values to match original test spec (共通/ポータル/初級 etc.)
</commit_message>
<xml_diff>
--- a/docs/テスト仕様書/テスト仕様書.xlsx
+++ b/docs/テスト仕様書/テスト仕様書.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="134">
   <si>
     <t>システム名</t>
   </si>
@@ -73,6 +73,9 @@
     <t>正常系</t>
   </si>
   <si>
+    <t>共通</t>
+  </si>
+  <si>
     <t>S-01</t>
   </si>
   <si>
@@ -133,6 +136,9 @@
     <t>ポータル画面へ戻り、ゲームの状態がリセットされる</t>
   </si>
   <si>
+    <t>ポータル</t>
+  </si>
+  <si>
     <t>P-01</t>
   </si>
   <si>
@@ -181,6 +187,9 @@
     <t>ポータル画面へ正しく戻る</t>
   </si>
   <si>
+    <t>初級</t>
+  </si>
+  <si>
     <t>B-01</t>
   </si>
   <si>
@@ -235,6 +244,9 @@
     <t>リザルト画面に「BRILLIANT!」クリアメッセージが表示される</t>
   </si>
   <si>
+    <t>通常</t>
+  </si>
+  <si>
     <t>N-01</t>
   </si>
   <si>
@@ -290,6 +302,9 @@
   </si>
   <si>
     <t>ボタンが薄くなり押しても何も起きない</t>
+  </si>
+  <si>
+    <t>上級</t>
   </si>
   <si>
     <t>E-01</t>
@@ -560,31 +575,31 @@
         <v>18</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -595,31 +610,31 @@
         <v>18</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
@@ -630,31 +645,31 @@
         <v>18</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11">
@@ -665,31 +680,31 @@
         <v>18</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12">
@@ -700,31 +715,31 @@
         <v>18</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13">
@@ -735,31 +750,31 @@
         <v>18</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14">
@@ -770,31 +785,31 @@
         <v>18</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15">
@@ -805,31 +820,31 @@
         <v>18</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16">
@@ -840,31 +855,31 @@
         <v>18</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17">
@@ -875,31 +890,31 @@
         <v>18</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18">
@@ -910,31 +925,31 @@
         <v>18</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19">
@@ -945,31 +960,31 @@
         <v>18</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20">
@@ -980,31 +995,31 @@
         <v>18</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21">
@@ -1015,31 +1030,31 @@
         <v>18</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22">
@@ -1050,31 +1065,31 @@
         <v>18</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23">
@@ -1085,31 +1100,31 @@
         <v>18</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24">
@@ -1120,31 +1135,31 @@
         <v>18</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25">
@@ -1155,31 +1170,31 @@
         <v>18</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26">
@@ -1190,31 +1205,31 @@
         <v>18</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="27">
@@ -1225,31 +1240,31 @@
         <v>18</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="28">
@@ -1257,34 +1272,34 @@
         <v>21</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K28" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="29">
@@ -1295,31 +1310,31 @@
         <v>18</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>18</v>
+        <v>96</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30">
@@ -1330,31 +1345,31 @@
         <v>18</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>18</v>
+        <v>96</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="31">
@@ -1365,31 +1380,31 @@
         <v>18</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>18</v>
+        <v>96</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32">
@@ -1400,31 +1415,31 @@
         <v>18</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>18</v>
+        <v>96</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="33">
@@ -1435,31 +1450,31 @@
         <v>18</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>18</v>
+        <v>96</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="34">
@@ -1470,31 +1485,31 @@
         <v>18</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>18</v>
+        <v>96</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="35">
@@ -1505,31 +1520,31 @@
         <v>18</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>18</v>
+        <v>96</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -1555,19 +1570,19 @@
         <v>7</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -1590,10 +1605,10 @@
         <v>11</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2">
@@ -1604,7 +1619,7 @@
         <v>18</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3">
@@ -1612,10 +1627,10 @@
         <v>8</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4">
@@ -1623,10 +1638,10 @@
         <v>8</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5">
@@ -1634,10 +1649,10 @@
         <v>14</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6">
@@ -1645,10 +1660,10 @@
         <v>14</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7">
@@ -1656,10 +1671,10 @@
         <v>14</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>